<commit_message>
Producao completa: livro Gratis Open Source + Playbook (V5 sem campanha/maquina)
- Livro 8 caps CONFORME: ~200k chars, 15 refs/cap, mermaid, artefatos tecnicos
- PDF: 98 paginas, 1003 KB (livro) + 365 KB (playbook)
- Auditoria R1-R15 + 5 gates F1/F2: OK
- Validar-codigo: 100% (17/17 blocos verificaveis)
- Subagentes free-program congelaram caps 5-8; escritos manualmente
- Mermaid-cli bloqueado por BOM no puppeteer config (problema local)

Entregas: livro_final.pdf, playbook.md/PDF, colecao sincronizada, pacote distribuicao
</commit_message>
<xml_diff>
--- a/rel-consumo/2026-08-20-consumo-cli.xlsx
+++ b/rel-consumo/2026-08-20-consumo-cli.xlsx
@@ -454,19 +454,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-08-20T14:50:00.229607+00:00</t>
+          <t>2026-08-20T14:49:59.738921+00:00</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-08-25T08:00:00.229625+00:00</t>
+          <t>2026-08-25T07:59:59.738942+00:00</t>
         </is>
       </c>
     </row>
@@ -723,22 +723,22 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>79791994</v>
+        <v>81655108</v>
       </c>
       <c r="E7" t="n">
-        <v>14344544</v>
+        <v>14413814</v>
       </c>
       <c r="F7" t="n">
-        <v>45943366</v>
+        <v>46036116</v>
       </c>
       <c r="G7" t="n">
-        <v>3601578826</v>
+        <v>3631313687</v>
       </c>
       <c r="H7" t="n">
-        <v>3744151719</v>
+        <v>3775911714</v>
       </c>
       <c r="I7" t="n">
-        <v>1035.1245</v>
+        <v>1038.8826</v>
       </c>
     </row>
   </sheetData>
@@ -3584,22 +3584,22 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>2153155</v>
+        <v>4182419</v>
       </c>
       <c r="E81" t="n">
-        <v>189684</v>
+        <v>259114</v>
       </c>
       <c r="F81" t="n">
-        <v>201778</v>
+        <v>294528</v>
       </c>
       <c r="G81" t="n">
-        <v>29616840</v>
+        <v>59352469</v>
       </c>
       <c r="H81" t="n">
-        <v>32166201</v>
+        <v>64093274</v>
       </c>
       <c r="I81" t="n">
-        <v>4.4508</v>
+        <v>8.2089</v>
       </c>
     </row>
   </sheetData>
@@ -4905,19 +4905,19 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>963103</v>
+        <v>2826097</v>
       </c>
       <c r="E37" t="n">
-        <v>47703</v>
+        <v>83577</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>6046976</v>
+        <v>20104352</v>
       </c>
       <c r="H37" t="n">
-        <v>7057892</v>
+        <v>23014136</v>
       </c>
       <c r="I37" t="n">
         <v>0</v>
@@ -8020,22 +8020,22 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>202</v>
+        <v>322</v>
       </c>
       <c r="E126" t="n">
-        <v>62203</v>
+        <v>95599</v>
       </c>
       <c r="F126" t="n">
-        <v>201778</v>
+        <v>294528</v>
       </c>
       <c r="G126" t="n">
-        <v>15106376</v>
+        <v>30783861</v>
       </c>
       <c r="H126" t="n">
-        <v>15370559</v>
+        <v>31174310</v>
       </c>
       <c r="I126" t="n">
-        <v>4.4508</v>
+        <v>8.2089</v>
       </c>
     </row>
     <row r="127">
@@ -38505,22 +38505,22 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>202</v>
+        <v>324</v>
       </c>
       <c r="E72" t="n">
-        <v>62203</v>
+        <v>97682</v>
       </c>
       <c r="F72" t="n">
-        <v>201778</v>
+        <v>297974</v>
       </c>
       <c r="G72" t="n">
-        <v>15106376</v>
+        <v>31062323</v>
       </c>
       <c r="H72" t="n">
-        <v>15370559</v>
+        <v>31458303</v>
       </c>
       <c r="I72" t="n">
-        <v>4.4508</v>
+        <v>8.299200000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>